<commit_message>
adding log complexity metrics and run the ablation for these metrics
</commit_message>
<xml_diff>
--- a/results/tables/compare/consolidated_results_tables_commitizen.xlsx
+++ b/results/tables/compare/consolidated_results_tables_commitizen.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://campusfl-my.sharepoint.com/personal/mahsa_choopannezhad_uni_li/Documents/Desktop/PhD materials/codes/Lifecycles-Processes/results/tables/commitizen/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://campusfl-my.sharepoint.com/personal/mahsa_choopannezhad_uni_li/Documents/Desktop/PhD materials/codes/Lifecycles-Processes/results/tables/compare/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="11_EB556F4FF53328B727DB86B233B6D209BADD7A48" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12FE7D04-9A34-415F-98D8-EF90CB897BD8}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="11_EB556F4FF53328B727DB86B233B6D209BADD7A48" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0A1DBBC-B067-46C3-B42C-2DC1D818BF43}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="41">
   <si>
     <t>log_name</t>
   </si>
@@ -155,6 +155,9 @@
   </si>
   <si>
     <t>wighted average</t>
+  </si>
+  <si>
+    <t>wighted average f score</t>
   </si>
 </sst>
 </file>
@@ -231,6 +234,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1817,10 +1824,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1864,7 +1874,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>26</v>
       </c>
@@ -1905,7 +1915,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -1946,7 +1956,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -1987,7 +1997,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -2028,7 +2038,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -2069,7 +2079,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -2110,7 +2120,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -2151,7 +2161,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -2192,7 +2202,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -2233,7 +2243,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -2280,10 +2290,10 @@
         <v>38</v>
       </c>
       <c r="P11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
@@ -2332,11 +2342,19 @@
         <v>0.58887864413577096</v>
       </c>
       <c r="P12" s="1">
-        <f>(C2*I2+C3*I3+C4*I4+C5*I5+C6*I6+C7*I7+C8*I8+C9*I9+C10*I10+C11*I11)/C12</f>
+        <f>($C$2*I2+$C$3*I3+$C$4*I4+$C$5*I5+$C$6*I6+$C$7*I7+$C$8*I8+$C$9*I9+$C$10*I10+$C$11*I11)/$C$12</f>
         <v>0.55309212385547502</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q12" s="1">
+        <f>($C$2*J2+$C$3*J3+$C$4*J4+$C$5*J5+$C$6*J6+$C$7*J7+$C$8*J8+$C$9*J9+$C$10*J10+$C$11*J11)/$C$12</f>
+        <v>713.69683544303803</v>
+      </c>
+      <c r="R12" s="1">
+        <f>($C$2*K2+$C$3*K3+$C$4*K4+$C$5*K5+$C$6*K6+$C$7*K7+$C$8*K8+$C$9*K9+$C$10*K10+$C$11*K11)/$C$12</f>
+        <v>45.999367088607592</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -2377,7 +2395,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -2418,7 +2436,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -2459,7 +2477,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -2500,7 +2518,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -2541,7 +2559,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -2582,7 +2600,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -2623,7 +2641,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -2664,7 +2682,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -2705,7 +2723,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -2755,7 +2773,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -2807,8 +2825,16 @@
         <f>(C13*I13+C14*I14+C15*I15+C16*I16+C17*I17+C18*I18+C19*I19+C20*I20+C21*I21+C22*I22)/C23</f>
         <v>0.48454808275306099</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q23" s="1">
+        <f>($C$2*J13+$C$3*J14+$C$4*J15+$C$5*J16+$C$6*J17+$C$7*J18+$C$8*J19+$C$9*J20+$C$10*J21+$C$11*J22)/$C$12</f>
+        <v>280.16392405063289</v>
+      </c>
+      <c r="R23" s="1">
+        <f>($C$2*K13+$C$3*K14+$C$4*K15+$C$5*K16+$C$6*K17+$C$7*K18+$C$8*K19+$C$9*K20+$C$10*K21+$C$11*K22)/$C$12</f>
+        <v>7.3746835443037977</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -2849,7 +2875,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -2890,7 +2916,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -2931,7 +2957,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>29</v>
       </c>
@@ -2972,7 +2998,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>30</v>
       </c>
@@ -3013,7 +3039,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>31</v>
       </c>
@@ -3054,7 +3080,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>32</v>
       </c>
@@ -3095,7 +3121,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>33</v>
       </c>
@@ -3136,7 +3162,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>34</v>
       </c>
@@ -3177,7 +3203,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>35</v>
       </c>
@@ -3227,7 +3253,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="34" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>21</v>
       </c>
@@ -3278,6 +3304,14 @@
       <c r="P34" s="1">
         <f>(C24*I24+C25*I25+C26*I26+C27*I27+C28*I28+C29*I29+C30*I30+C31*I31+C32*I32+C33*I33)/C34</f>
         <v>0.59338217803243765</v>
+      </c>
+      <c r="Q34" s="1">
+        <f>($C$2*J24+$C$3*J25+$C$4*J26+$C$5*J27+$C$6*J28+$C$7*J29+$C$8*J30+$C$9*J31+$C$10*J32+$C$11*J33)/$C$12</f>
+        <v>417.3</v>
+      </c>
+      <c r="R34" s="1">
+        <f>($C$2*K24+$C$3*K25+$C$4*K26+$C$5*K27+$C$6*K28+$C$7*K29+$C$8*K30+$C$9*K31+$C$10*K32+$C$11*K33)/$C$12</f>
+        <v>50.860126582278482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>